<commit_message>
fix: Auditoria minuciosa y vinculacion exacta de 245 imagenes existentes para el catalogo completo
</commit_message>
<xml_diff>
--- a/INVENTARIO HALLOWEEN (3).xlsx
+++ b/INVENTARIO HALLOWEEN (3).xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="985" uniqueCount="419">
   <si>
     <t>CODIGO</t>
   </si>
@@ -766,72 +766,6 @@
     <t>DIS-0245</t>
   </si>
   <si>
-    <t>DIS-0246</t>
-  </si>
-  <si>
-    <t>DIS-0247</t>
-  </si>
-  <si>
-    <t>DIS-0248</t>
-  </si>
-  <si>
-    <t>DIS-0249</t>
-  </si>
-  <si>
-    <t>DIS-0250</t>
-  </si>
-  <si>
-    <t>DIS-0251</t>
-  </si>
-  <si>
-    <t>DIS-0252</t>
-  </si>
-  <si>
-    <t>DIS-0253</t>
-  </si>
-  <si>
-    <t>DIS-0254</t>
-  </si>
-  <si>
-    <t>DIS-0255</t>
-  </si>
-  <si>
-    <t>DIS-0256</t>
-  </si>
-  <si>
-    <t>DIS-0257</t>
-  </si>
-  <si>
-    <t>DIS-0258</t>
-  </si>
-  <si>
-    <t>DIS-0259</t>
-  </si>
-  <si>
-    <t>DIS-0260</t>
-  </si>
-  <si>
-    <t>DIS-0261</t>
-  </si>
-  <si>
-    <t>DIS-0262</t>
-  </si>
-  <si>
-    <t>DIS-0263</t>
-  </si>
-  <si>
-    <t>DIS-0264</t>
-  </si>
-  <si>
-    <t>DIS-0265</t>
-  </si>
-  <si>
-    <t>DIS-0266</t>
-  </si>
-  <si>
-    <t>DIS-0267</t>
-  </si>
-  <si>
     <t>CHINA</t>
   </si>
   <si>
@@ -1276,9 +1210,6 @@
     <t>BAILARINA AZUL</t>
   </si>
   <si>
-    <t>nan</t>
-  </si>
-  <si>
     <t>S</t>
   </si>
   <si>
@@ -1340,9 +1271,6 @@
   </si>
   <si>
     <t>NIÑO</t>
-  </si>
-  <si>
-    <t>NAN</t>
   </si>
 </sst>
 </file>
@@ -1674,7 +1602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E268"/>
+  <dimension ref="A1:E246"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1699,13 +1627,13 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>272</v>
+        <v>250</v>
       </c>
       <c r="C2" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D2" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E2">
         <v>5000</v>
@@ -1716,13 +1644,13 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>273</v>
+        <v>251</v>
       </c>
       <c r="C3" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D3" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E3">
         <v>10000</v>
@@ -1733,13 +1661,13 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="C4" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D4" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E4">
         <v>10000</v>
@@ -1750,13 +1678,13 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>275</v>
+        <v>253</v>
       </c>
       <c r="C5" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D5" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E5">
         <v>5000</v>
@@ -1767,13 +1695,13 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>276</v>
+        <v>254</v>
       </c>
       <c r="C6" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D6" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E6">
         <v>7000</v>
@@ -1784,13 +1712,13 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="C7" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D7" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E7">
         <v>5000</v>
@@ -1801,13 +1729,13 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>278</v>
+        <v>256</v>
       </c>
       <c r="C8" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D8" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E8">
         <v>4000</v>
@@ -1818,13 +1746,13 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>279</v>
+        <v>257</v>
       </c>
       <c r="C9" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D9" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E9">
         <v>10000</v>
@@ -1835,13 +1763,13 @@
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="C10" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D10" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E10">
         <v>7000</v>
@@ -1852,13 +1780,13 @@
         <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="C11" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D11" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E11">
         <v>5000</v>
@@ -1869,13 +1797,13 @@
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="C12" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D12" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E12">
         <v>7000</v>
@@ -1886,13 +1814,13 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>283</v>
+        <v>261</v>
       </c>
       <c r="C13" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D13" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E13">
         <v>7000</v>
@@ -1903,13 +1831,13 @@
         <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>284</v>
+        <v>262</v>
       </c>
       <c r="C14" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D14" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E14">
         <v>5000</v>
@@ -1920,13 +1848,13 @@
         <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="C15" t="s">
-        <v>425</v>
+        <v>402</v>
       </c>
       <c r="D15" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E15">
         <v>7000</v>
@@ -1937,13 +1865,13 @@
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="C16" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D16" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E16">
         <v>4000</v>
@@ -1954,13 +1882,13 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="C17" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D17" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E17">
         <v>5000</v>
@@ -1971,13 +1899,13 @@
         <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>288</v>
+        <v>266</v>
       </c>
       <c r="C18" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D18" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E18">
         <v>7000</v>
@@ -1988,13 +1916,13 @@
         <v>22</v>
       </c>
       <c r="B19" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="C19" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D19" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E19">
         <v>5000</v>
@@ -2005,13 +1933,13 @@
         <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>290</v>
+        <v>268</v>
       </c>
       <c r="C20" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D20" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E20">
         <v>4000</v>
@@ -2022,13 +1950,13 @@
         <v>24</v>
       </c>
       <c r="B21" t="s">
-        <v>291</v>
+        <v>269</v>
       </c>
       <c r="C21" t="s">
-        <v>425</v>
+        <v>402</v>
       </c>
       <c r="D21" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E21">
         <v>7000</v>
@@ -2039,13 +1967,13 @@
         <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>292</v>
+        <v>270</v>
       </c>
       <c r="C22" t="s">
-        <v>425</v>
+        <v>402</v>
       </c>
       <c r="D22" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E22">
         <v>8000</v>
@@ -2056,13 +1984,13 @@
         <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>293</v>
+        <v>271</v>
       </c>
       <c r="C23" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D23" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E23">
         <v>8000</v>
@@ -2073,13 +2001,13 @@
         <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>294</v>
+        <v>272</v>
       </c>
       <c r="C24" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D24" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E24">
         <v>5000</v>
@@ -2090,13 +2018,13 @@
         <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>295</v>
+        <v>273</v>
       </c>
       <c r="C25" t="s">
-        <v>428</v>
+        <v>405</v>
       </c>
       <c r="D25" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E25">
         <v>8000</v>
@@ -2107,13 +2035,13 @@
         <v>29</v>
       </c>
       <c r="B26" t="s">
-        <v>296</v>
+        <v>274</v>
       </c>
       <c r="C26" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D26" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E26">
         <v>5000</v>
@@ -2124,13 +2052,13 @@
         <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>297</v>
+        <v>275</v>
       </c>
       <c r="C27" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D27" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E27">
         <v>7000</v>
@@ -2141,13 +2069,13 @@
         <v>31</v>
       </c>
       <c r="B28" t="s">
-        <v>298</v>
+        <v>276</v>
       </c>
       <c r="C28" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D28" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E28">
         <v>5000</v>
@@ -2158,13 +2086,13 @@
         <v>32</v>
       </c>
       <c r="B29" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="C29" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D29" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E29">
         <v>5000</v>
@@ -2175,13 +2103,13 @@
         <v>33</v>
       </c>
       <c r="B30" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="C30" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D30" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E30">
         <v>5000</v>
@@ -2192,13 +2120,13 @@
         <v>34</v>
       </c>
       <c r="B31" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="C31" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D31" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E31">
         <v>5000</v>
@@ -2209,13 +2137,13 @@
         <v>35</v>
       </c>
       <c r="B32" t="s">
-        <v>300</v>
+        <v>278</v>
       </c>
       <c r="C32" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D32" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E32">
         <v>8000</v>
@@ -2226,13 +2154,13 @@
         <v>36</v>
       </c>
       <c r="B33" t="s">
-        <v>301</v>
+        <v>279</v>
       </c>
       <c r="C33" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D33" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E33">
         <v>7000</v>
@@ -2243,13 +2171,13 @@
         <v>37</v>
       </c>
       <c r="B34" t="s">
-        <v>302</v>
+        <v>280</v>
       </c>
       <c r="C34" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D34" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E34">
         <v>8000</v>
@@ -2260,13 +2188,13 @@
         <v>38</v>
       </c>
       <c r="B35" t="s">
-        <v>303</v>
+        <v>281</v>
       </c>
       <c r="C35" t="s">
-        <v>431</v>
+        <v>408</v>
       </c>
       <c r="D35" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E35">
         <v>5000</v>
@@ -2277,13 +2205,13 @@
         <v>39</v>
       </c>
       <c r="B36" t="s">
-        <v>304</v>
+        <v>282</v>
       </c>
       <c r="C36" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="D36" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E36">
         <v>5000</v>
@@ -2294,13 +2222,13 @@
         <v>40</v>
       </c>
       <c r="B37" t="s">
-        <v>305</v>
+        <v>283</v>
       </c>
       <c r="C37" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="D37" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E37">
         <v>5000</v>
@@ -2311,13 +2239,13 @@
         <v>41</v>
       </c>
       <c r="B38" t="s">
-        <v>306</v>
+        <v>284</v>
       </c>
       <c r="C38" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D38" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E38">
         <v>5000</v>
@@ -2328,13 +2256,13 @@
         <v>42</v>
       </c>
       <c r="B39" t="s">
-        <v>307</v>
+        <v>285</v>
       </c>
       <c r="C39" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D39" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E39">
         <v>5000</v>
@@ -2345,13 +2273,13 @@
         <v>43</v>
       </c>
       <c r="B40" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="C40" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D40" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E40">
         <v>5000</v>
@@ -2362,13 +2290,13 @@
         <v>44</v>
       </c>
       <c r="B41" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="C41" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D41" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E41">
         <v>5000</v>
@@ -2379,13 +2307,13 @@
         <v>45</v>
       </c>
       <c r="B42" t="s">
-        <v>308</v>
+        <v>286</v>
       </c>
       <c r="C42" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D42" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E42">
         <v>7000</v>
@@ -2396,13 +2324,13 @@
         <v>46</v>
       </c>
       <c r="B43" t="s">
-        <v>309</v>
+        <v>287</v>
       </c>
       <c r="C43" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D43" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E43">
         <v>5000</v>
@@ -2413,13 +2341,13 @@
         <v>47</v>
       </c>
       <c r="B44" t="s">
-        <v>310</v>
+        <v>288</v>
       </c>
       <c r="C44" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D44" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E44">
         <v>10000</v>
@@ -2430,13 +2358,13 @@
         <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>311</v>
+        <v>289</v>
       </c>
       <c r="C45" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D45" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E45">
         <v>7000</v>
@@ -2447,13 +2375,13 @@
         <v>49</v>
       </c>
       <c r="B46" t="s">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="C46" t="s">
-        <v>431</v>
+        <v>408</v>
       </c>
       <c r="D46" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E46">
         <v>10000</v>
@@ -2464,13 +2392,13 @@
         <v>50</v>
       </c>
       <c r="B47" t="s">
-        <v>313</v>
+        <v>291</v>
       </c>
       <c r="C47" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D47" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E47">
         <v>10000</v>
@@ -2481,13 +2409,13 @@
         <v>51</v>
       </c>
       <c r="B48" t="s">
-        <v>308</v>
+        <v>286</v>
       </c>
       <c r="C48" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D48" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E48">
         <v>7000</v>
@@ -2498,13 +2426,13 @@
         <v>52</v>
       </c>
       <c r="B49" t="s">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="C49" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D49" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E49">
         <v>10000</v>
@@ -2515,13 +2443,13 @@
         <v>53</v>
       </c>
       <c r="B50" t="s">
-        <v>314</v>
+        <v>292</v>
       </c>
       <c r="C50" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D50" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E50">
         <v>7000</v>
@@ -2532,13 +2460,13 @@
         <v>54</v>
       </c>
       <c r="B51" t="s">
-        <v>315</v>
+        <v>293</v>
       </c>
       <c r="C51" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D51" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E51">
         <v>5000</v>
@@ -2549,13 +2477,13 @@
         <v>55</v>
       </c>
       <c r="B52" t="s">
-        <v>316</v>
+        <v>294</v>
       </c>
       <c r="C52" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D52" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E52">
         <v>7000</v>
@@ -2566,13 +2494,13 @@
         <v>56</v>
       </c>
       <c r="B53" t="s">
-        <v>317</v>
+        <v>295</v>
       </c>
       <c r="C53" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D53" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E53">
         <v>5000</v>
@@ -2583,13 +2511,13 @@
         <v>57</v>
       </c>
       <c r="B54" t="s">
-        <v>318</v>
+        <v>296</v>
       </c>
       <c r="C54" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D54" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E54">
         <v>5000</v>
@@ -2600,13 +2528,13 @@
         <v>58</v>
       </c>
       <c r="B55" t="s">
-        <v>319</v>
+        <v>297</v>
       </c>
       <c r="C55" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D55" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E55">
         <v>8000</v>
@@ -2617,13 +2545,13 @@
         <v>59</v>
       </c>
       <c r="B56" t="s">
-        <v>320</v>
+        <v>298</v>
       </c>
       <c r="C56" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D56" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E56">
         <v>7000</v>
@@ -2634,13 +2562,13 @@
         <v>60</v>
       </c>
       <c r="B57" t="s">
-        <v>321</v>
+        <v>299</v>
       </c>
       <c r="C57" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D57" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E57">
         <v>10000</v>
@@ -2651,13 +2579,13 @@
         <v>61</v>
       </c>
       <c r="B58" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="C58" t="s">
-        <v>435</v>
+        <v>412</v>
       </c>
       <c r="D58" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E58">
         <v>5000</v>
@@ -2668,13 +2596,13 @@
         <v>62</v>
       </c>
       <c r="B59" t="s">
-        <v>322</v>
+        <v>300</v>
       </c>
       <c r="C59" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D59" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E59">
         <v>8000</v>
@@ -2685,13 +2613,13 @@
         <v>63</v>
       </c>
       <c r="B60" t="s">
-        <v>323</v>
+        <v>301</v>
       </c>
       <c r="C60" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D60" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E60">
         <v>5000</v>
@@ -2702,13 +2630,13 @@
         <v>64</v>
       </c>
       <c r="B61" t="s">
-        <v>324</v>
+        <v>302</v>
       </c>
       <c r="C61" t="s">
-        <v>436</v>
+        <v>413</v>
       </c>
       <c r="D61" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E61">
         <v>5000</v>
@@ -2719,13 +2647,13 @@
         <v>65</v>
       </c>
       <c r="B62" t="s">
-        <v>324</v>
+        <v>302</v>
       </c>
       <c r="C62" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D62" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E62">
         <v>5000</v>
@@ -2736,13 +2664,13 @@
         <v>66</v>
       </c>
       <c r="B63" t="s">
-        <v>325</v>
+        <v>303</v>
       </c>
       <c r="C63" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D63" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E63">
         <v>8000</v>
@@ -2753,13 +2681,13 @@
         <v>67</v>
       </c>
       <c r="B64" t="s">
-        <v>326</v>
+        <v>304</v>
       </c>
       <c r="C64" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D64" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E64">
         <v>8000</v>
@@ -2770,13 +2698,13 @@
         <v>68</v>
       </c>
       <c r="B65" t="s">
-        <v>327</v>
+        <v>305</v>
       </c>
       <c r="C65" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D65" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E65">
         <v>5000</v>
@@ -2787,13 +2715,13 @@
         <v>69</v>
       </c>
       <c r="B66" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="C66" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D66" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E66">
         <v>5000</v>
@@ -2804,13 +2732,13 @@
         <v>70</v>
       </c>
       <c r="B67" t="s">
-        <v>328</v>
+        <v>306</v>
       </c>
       <c r="C67" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D67" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E67">
         <v>8000</v>
@@ -2821,13 +2749,13 @@
         <v>71</v>
       </c>
       <c r="B68" t="s">
-        <v>298</v>
+        <v>276</v>
       </c>
       <c r="C68" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D68" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E68">
         <v>5000</v>
@@ -2838,13 +2766,13 @@
         <v>72</v>
       </c>
       <c r="B69" t="s">
-        <v>329</v>
+        <v>307</v>
       </c>
       <c r="C69" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D69" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E69">
         <v>5000</v>
@@ -2855,13 +2783,13 @@
         <v>73</v>
       </c>
       <c r="B70" t="s">
-        <v>330</v>
+        <v>308</v>
       </c>
       <c r="C70" t="s">
-        <v>437</v>
+        <v>414</v>
       </c>
       <c r="D70" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E70">
         <v>5000</v>
@@ -2872,13 +2800,13 @@
         <v>74</v>
       </c>
       <c r="B71" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="C71" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D71" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E71">
         <v>8000</v>
@@ -2889,13 +2817,13 @@
         <v>75</v>
       </c>
       <c r="B72" t="s">
-        <v>331</v>
+        <v>309</v>
       </c>
       <c r="C72" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D72" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E72">
         <v>7000</v>
@@ -2906,13 +2834,13 @@
         <v>76</v>
       </c>
       <c r="B73" t="s">
-        <v>308</v>
+        <v>286</v>
       </c>
       <c r="C73" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D73" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E73">
         <v>7000</v>
@@ -2923,13 +2851,13 @@
         <v>77</v>
       </c>
       <c r="B74" t="s">
-        <v>332</v>
+        <v>310</v>
       </c>
       <c r="C74" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D74" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E74">
         <v>5000</v>
@@ -2940,13 +2868,13 @@
         <v>78</v>
       </c>
       <c r="B75" t="s">
-        <v>333</v>
+        <v>311</v>
       </c>
       <c r="C75" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D75" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E75">
         <v>5000</v>
@@ -2957,13 +2885,13 @@
         <v>79</v>
       </c>
       <c r="B76" t="s">
-        <v>323</v>
+        <v>301</v>
       </c>
       <c r="C76" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D76" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E76">
         <v>5000</v>
@@ -2974,13 +2902,13 @@
         <v>80</v>
       </c>
       <c r="B77" t="s">
-        <v>334</v>
+        <v>312</v>
       </c>
       <c r="C77" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D77" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E77">
         <v>5000</v>
@@ -2991,13 +2919,13 @@
         <v>81</v>
       </c>
       <c r="B78" t="s">
-        <v>335</v>
+        <v>313</v>
       </c>
       <c r="C78" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D78" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E78">
         <v>5000</v>
@@ -3008,13 +2936,13 @@
         <v>82</v>
       </c>
       <c r="B79" t="s">
-        <v>336</v>
+        <v>314</v>
       </c>
       <c r="C79" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D79" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E79">
         <v>5000</v>
@@ -3025,13 +2953,13 @@
         <v>83</v>
       </c>
       <c r="B80" t="s">
-        <v>337</v>
+        <v>315</v>
       </c>
       <c r="C80" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D80" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E80">
         <v>8000</v>
@@ -3042,13 +2970,13 @@
         <v>84</v>
       </c>
       <c r="B81" t="s">
-        <v>310</v>
+        <v>288</v>
       </c>
       <c r="C81" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="D81" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E81">
         <v>5000</v>
@@ -3059,13 +2987,13 @@
         <v>85</v>
       </c>
       <c r="B82" t="s">
-        <v>338</v>
+        <v>316</v>
       </c>
       <c r="C82" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D82" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E82">
         <v>7000</v>
@@ -3076,13 +3004,13 @@
         <v>86</v>
       </c>
       <c r="B83" t="s">
-        <v>320</v>
+        <v>298</v>
       </c>
       <c r="C83" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D83" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E83">
         <v>5000</v>
@@ -3093,13 +3021,13 @@
         <v>87</v>
       </c>
       <c r="B84" t="s">
-        <v>327</v>
+        <v>305</v>
       </c>
       <c r="C84" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D84" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E84">
         <v>7000</v>
@@ -3110,13 +3038,13 @@
         <v>88</v>
       </c>
       <c r="B85" t="s">
-        <v>339</v>
+        <v>317</v>
       </c>
       <c r="C85" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D85" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E85">
         <v>7000</v>
@@ -3127,13 +3055,13 @@
         <v>89</v>
       </c>
       <c r="B86" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="C86" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D86" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E86">
         <v>7000</v>
@@ -3144,13 +3072,13 @@
         <v>90</v>
       </c>
       <c r="B87" t="s">
-        <v>340</v>
+        <v>318</v>
       </c>
       <c r="C87" t="s">
-        <v>437</v>
+        <v>414</v>
       </c>
       <c r="D87" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E87">
         <v>5000</v>
@@ -3161,13 +3089,13 @@
         <v>91</v>
       </c>
       <c r="B88" t="s">
-        <v>341</v>
+        <v>319</v>
       </c>
       <c r="C88" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D88" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E88">
         <v>5000</v>
@@ -3178,13 +3106,13 @@
         <v>92</v>
       </c>
       <c r="B89" t="s">
-        <v>342</v>
+        <v>320</v>
       </c>
       <c r="C89" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D89" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E89">
         <v>5000</v>
@@ -3195,13 +3123,13 @@
         <v>93</v>
       </c>
       <c r="B90" t="s">
-        <v>343</v>
+        <v>321</v>
       </c>
       <c r="C90" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D90" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E90">
         <v>8000</v>
@@ -3212,13 +3140,13 @@
         <v>94</v>
       </c>
       <c r="B91" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="C91" t="s">
-        <v>436</v>
+        <v>413</v>
       </c>
       <c r="D91" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E91">
         <v>7000</v>
@@ -3229,13 +3157,13 @@
         <v>95</v>
       </c>
       <c r="B92" t="s">
-        <v>344</v>
+        <v>322</v>
       </c>
       <c r="C92" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="D92" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E92">
         <v>5000</v>
@@ -3246,13 +3174,13 @@
         <v>96</v>
       </c>
       <c r="B93" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C93" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="D93" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E93">
         <v>7000</v>
@@ -3263,13 +3191,13 @@
         <v>97</v>
       </c>
       <c r="B94" t="s">
-        <v>346</v>
+        <v>324</v>
       </c>
       <c r="C94" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D94" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E94">
         <v>5000</v>
@@ -3280,13 +3208,13 @@
         <v>98</v>
       </c>
       <c r="B95" t="s">
-        <v>347</v>
+        <v>325</v>
       </c>
       <c r="C95" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D95" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E95">
         <v>10000</v>
@@ -3297,13 +3225,13 @@
         <v>99</v>
       </c>
       <c r="B96" t="s">
-        <v>348</v>
+        <v>326</v>
       </c>
       <c r="C96" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D96" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E96">
         <v>5000</v>
@@ -3314,13 +3242,13 @@
         <v>100</v>
       </c>
       <c r="B97" t="s">
-        <v>349</v>
+        <v>327</v>
       </c>
       <c r="C97" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D97" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E97">
         <v>5000</v>
@@ -3331,13 +3259,13 @@
         <v>101</v>
       </c>
       <c r="B98" t="s">
-        <v>331</v>
+        <v>309</v>
       </c>
       <c r="C98" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D98" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E98">
         <v>5000</v>
@@ -3348,13 +3276,13 @@
         <v>102</v>
       </c>
       <c r="B99" t="s">
-        <v>350</v>
+        <v>328</v>
       </c>
       <c r="C99" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D99" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E99">
         <v>7000</v>
@@ -3365,13 +3293,13 @@
         <v>103</v>
       </c>
       <c r="B100" t="s">
-        <v>351</v>
+        <v>329</v>
       </c>
       <c r="C100" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D100" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E100">
         <v>7000</v>
@@ -3382,13 +3310,13 @@
         <v>104</v>
       </c>
       <c r="B101" t="s">
-        <v>328</v>
+        <v>306</v>
       </c>
       <c r="C101" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D101" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E101">
         <v>5000</v>
@@ -3399,13 +3327,13 @@
         <v>105</v>
       </c>
       <c r="B102" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="C102" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D102" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E102">
         <v>5000</v>
@@ -3416,13 +3344,13 @@
         <v>106</v>
       </c>
       <c r="B103" t="s">
-        <v>352</v>
+        <v>330</v>
       </c>
       <c r="C103" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D103" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E103">
         <v>8000</v>
@@ -3433,13 +3361,13 @@
         <v>107</v>
       </c>
       <c r="B104" t="s">
-        <v>353</v>
+        <v>331</v>
       </c>
       <c r="C104" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D104" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E104">
         <v>7000</v>
@@ -3450,13 +3378,13 @@
         <v>108</v>
       </c>
       <c r="B105" t="s">
-        <v>354</v>
+        <v>332</v>
       </c>
       <c r="C105" t="s">
-        <v>436</v>
+        <v>413</v>
       </c>
       <c r="D105" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E105">
         <v>5000</v>
@@ -3467,13 +3395,13 @@
         <v>109</v>
       </c>
       <c r="B106" t="s">
-        <v>355</v>
+        <v>333</v>
       </c>
       <c r="C106" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D106" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E106">
         <v>5000</v>
@@ -3484,13 +3412,13 @@
         <v>110</v>
       </c>
       <c r="B107" t="s">
-        <v>294</v>
+        <v>272</v>
       </c>
       <c r="C107" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D107" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E107">
         <v>5000</v>
@@ -3501,13 +3429,13 @@
         <v>111</v>
       </c>
       <c r="B108" t="s">
-        <v>352</v>
+        <v>330</v>
       </c>
       <c r="C108" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D108" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E108">
         <v>5000</v>
@@ -3518,13 +3446,13 @@
         <v>112</v>
       </c>
       <c r="B109" t="s">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="C109" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D109" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E109">
         <v>5000</v>
@@ -3535,13 +3463,13 @@
         <v>113</v>
       </c>
       <c r="B110" t="s">
-        <v>321</v>
+        <v>299</v>
       </c>
       <c r="C110" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D110" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E110">
         <v>5000</v>
@@ -3552,13 +3480,13 @@
         <v>114</v>
       </c>
       <c r="B111" t="s">
-        <v>356</v>
+        <v>334</v>
       </c>
       <c r="C111" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D111" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E111">
         <v>5000</v>
@@ -3569,13 +3497,13 @@
         <v>115</v>
       </c>
       <c r="B112" t="s">
-        <v>335</v>
+        <v>313</v>
       </c>
       <c r="C112" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="D112" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E112">
         <v>5000</v>
@@ -3586,13 +3514,13 @@
         <v>116</v>
       </c>
       <c r="B113" t="s">
-        <v>357</v>
+        <v>335</v>
       </c>
       <c r="C113" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D113" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E113">
         <v>5000</v>
@@ -3603,13 +3531,13 @@
         <v>117</v>
       </c>
       <c r="B114" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="C114" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D114" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E114">
         <v>5000</v>
@@ -3620,13 +3548,13 @@
         <v>118</v>
       </c>
       <c r="B115" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="C115" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D115" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E115">
         <v>5000</v>
@@ -3637,13 +3565,13 @@
         <v>119</v>
       </c>
       <c r="B116" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="C116" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D116" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E116">
         <v>5000</v>
@@ -3654,13 +3582,13 @@
         <v>120</v>
       </c>
       <c r="B117" t="s">
-        <v>352</v>
+        <v>330</v>
       </c>
       <c r="C117" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D117" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E117">
         <v>5000</v>
@@ -3671,13 +3599,13 @@
         <v>121</v>
       </c>
       <c r="B118" t="s">
-        <v>317</v>
+        <v>295</v>
       </c>
       <c r="C118" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D118" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E118">
         <v>5000</v>
@@ -3688,13 +3616,13 @@
         <v>122</v>
       </c>
       <c r="B119" t="s">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="C119" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D119" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E119">
         <v>5000</v>
@@ -3705,13 +3633,13 @@
         <v>123</v>
       </c>
       <c r="B120" t="s">
-        <v>340</v>
+        <v>318</v>
       </c>
       <c r="C120" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D120" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E120">
         <v>5000</v>
@@ -3722,13 +3650,13 @@
         <v>124</v>
       </c>
       <c r="B121" t="s">
-        <v>358</v>
+        <v>336</v>
       </c>
       <c r="C121" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D121" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E121">
         <v>7000</v>
@@ -3739,13 +3667,13 @@
         <v>125</v>
       </c>
       <c r="B122" t="s">
-        <v>311</v>
+        <v>289</v>
       </c>
       <c r="C122" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D122" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E122">
         <v>5000</v>
@@ -3756,13 +3684,13 @@
         <v>126</v>
       </c>
       <c r="B123" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C123" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D123" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E123">
         <v>7000</v>
@@ -3773,13 +3701,13 @@
         <v>127</v>
       </c>
       <c r="B124" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C124" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D124" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E124">
         <v>7000</v>
@@ -3790,13 +3718,13 @@
         <v>128</v>
       </c>
       <c r="B125" t="s">
-        <v>339</v>
+        <v>317</v>
       </c>
       <c r="C125" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D125" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E125">
         <v>7000</v>
@@ -3807,13 +3735,13 @@
         <v>129</v>
       </c>
       <c r="B126" t="s">
-        <v>359</v>
+        <v>337</v>
       </c>
       <c r="C126" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D126" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E126">
         <v>5000</v>
@@ -3824,13 +3752,13 @@
         <v>130</v>
       </c>
       <c r="B127" t="s">
-        <v>360</v>
+        <v>338</v>
       </c>
       <c r="C127" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D127" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E127">
         <v>5000</v>
@@ -3841,13 +3769,13 @@
         <v>131</v>
       </c>
       <c r="B128" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C128" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D128" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E128">
         <v>10000</v>
@@ -3858,13 +3786,13 @@
         <v>132</v>
       </c>
       <c r="B129" t="s">
-        <v>331</v>
+        <v>309</v>
       </c>
       <c r="C129" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D129" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E129">
         <v>5000</v>
@@ -3875,13 +3803,13 @@
         <v>133</v>
       </c>
       <c r="B130" t="s">
-        <v>361</v>
+        <v>339</v>
       </c>
       <c r="C130" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D130" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E130">
         <v>5000</v>
@@ -3892,13 +3820,13 @@
         <v>134</v>
       </c>
       <c r="B131" t="s">
-        <v>362</v>
+        <v>340</v>
       </c>
       <c r="C131" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D131" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E131">
         <v>5000</v>
@@ -3909,13 +3837,13 @@
         <v>135</v>
       </c>
       <c r="B132" t="s">
-        <v>308</v>
+        <v>286</v>
       </c>
       <c r="C132" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D132" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E132">
         <v>7000</v>
@@ -3926,13 +3854,13 @@
         <v>136</v>
       </c>
       <c r="B133" t="s">
-        <v>363</v>
+        <v>341</v>
       </c>
       <c r="C133" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D133" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E133">
         <v>5000</v>
@@ -3943,13 +3871,13 @@
         <v>137</v>
       </c>
       <c r="B134" t="s">
-        <v>339</v>
+        <v>317</v>
       </c>
       <c r="C134" t="s">
-        <v>437</v>
+        <v>414</v>
       </c>
       <c r="D134" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E134">
         <v>8000</v>
@@ -3960,13 +3888,13 @@
         <v>138</v>
       </c>
       <c r="B135" t="s">
-        <v>364</v>
+        <v>342</v>
       </c>
       <c r="C135" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="D135" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E135">
         <v>5000</v>
@@ -3977,13 +3905,13 @@
         <v>139</v>
       </c>
       <c r="B136" t="s">
-        <v>365</v>
+        <v>343</v>
       </c>
       <c r="C136" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D136" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E136">
         <v>7000</v>
@@ -3994,13 +3922,13 @@
         <v>140</v>
       </c>
       <c r="B137" t="s">
-        <v>339</v>
+        <v>317</v>
       </c>
       <c r="C137" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D137" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E137">
         <v>10000</v>
@@ -4011,13 +3939,13 @@
         <v>141</v>
       </c>
       <c r="B138" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C138" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D138" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E138">
         <v>8000</v>
@@ -4028,13 +3956,13 @@
         <v>142</v>
       </c>
       <c r="B139" t="s">
-        <v>366</v>
+        <v>344</v>
       </c>
       <c r="C139" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D139" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E139">
         <v>10000</v>
@@ -4045,13 +3973,13 @@
         <v>143</v>
       </c>
       <c r="B140" t="s">
-        <v>367</v>
+        <v>345</v>
       </c>
       <c r="C140" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D140" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E140">
         <v>10000</v>
@@ -4062,13 +3990,13 @@
         <v>144</v>
       </c>
       <c r="B141" t="s">
-        <v>368</v>
+        <v>346</v>
       </c>
       <c r="C141" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D141" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E141">
         <v>7000</v>
@@ -4079,13 +4007,13 @@
         <v>145</v>
       </c>
       <c r="B142" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C142" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D142" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E142">
         <v>7000</v>
@@ -4096,13 +4024,13 @@
         <v>146</v>
       </c>
       <c r="B143" t="s">
-        <v>320</v>
+        <v>298</v>
       </c>
       <c r="C143" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D143" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E143">
         <v>5000</v>
@@ -4113,13 +4041,13 @@
         <v>147</v>
       </c>
       <c r="B144" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C144" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D144" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E144">
         <v>5000</v>
@@ -4130,13 +4058,13 @@
         <v>148</v>
       </c>
       <c r="B145" t="s">
-        <v>308</v>
+        <v>286</v>
       </c>
       <c r="C145" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D145" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E145">
         <v>5000</v>
@@ -4147,13 +4075,13 @@
         <v>149</v>
       </c>
       <c r="B146" t="s">
-        <v>338</v>
+        <v>316</v>
       </c>
       <c r="C146" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D146" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E146">
         <v>5000</v>
@@ -4164,13 +4092,13 @@
         <v>150</v>
       </c>
       <c r="B147" t="s">
-        <v>315</v>
+        <v>293</v>
       </c>
       <c r="C147" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D147" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E147">
         <v>5000</v>
@@ -4181,13 +4109,13 @@
         <v>151</v>
       </c>
       <c r="B148" t="s">
-        <v>349</v>
+        <v>327</v>
       </c>
       <c r="C148" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D148" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E148">
         <v>5000</v>
@@ -4198,13 +4126,13 @@
         <v>152</v>
       </c>
       <c r="B149" t="s">
-        <v>369</v>
+        <v>347</v>
       </c>
       <c r="C149" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D149" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E149">
         <v>7000</v>
@@ -4215,13 +4143,13 @@
         <v>153</v>
       </c>
       <c r="B150" t="s">
-        <v>370</v>
+        <v>348</v>
       </c>
       <c r="C150" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D150" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E150">
         <v>10000</v>
@@ -4232,13 +4160,13 @@
         <v>154</v>
       </c>
       <c r="B151" t="s">
-        <v>371</v>
+        <v>349</v>
       </c>
       <c r="C151" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D151" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E151">
         <v>7000</v>
@@ -4249,13 +4177,13 @@
         <v>155</v>
       </c>
       <c r="B152" t="s">
-        <v>372</v>
+        <v>350</v>
       </c>
       <c r="C152" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="D152" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E152">
         <v>7000</v>
@@ -4266,13 +4194,13 @@
         <v>156</v>
       </c>
       <c r="B153" t="s">
-        <v>373</v>
+        <v>351</v>
       </c>
       <c r="C153" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D153" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E153">
         <v>7000</v>
@@ -4283,13 +4211,13 @@
         <v>157</v>
       </c>
       <c r="B154" t="s">
-        <v>338</v>
+        <v>316</v>
       </c>
       <c r="C154" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D154" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E154">
         <v>7000</v>
@@ -4300,13 +4228,13 @@
         <v>158</v>
       </c>
       <c r="B155" t="s">
-        <v>374</v>
+        <v>352</v>
       </c>
       <c r="C155" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D155" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E155">
         <v>8000</v>
@@ -4317,13 +4245,13 @@
         <v>159</v>
       </c>
       <c r="B156" t="s">
-        <v>328</v>
+        <v>306</v>
       </c>
       <c r="C156" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D156" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E156">
         <v>5000</v>
@@ -4334,13 +4262,13 @@
         <v>160</v>
       </c>
       <c r="B157" t="s">
-        <v>348</v>
+        <v>326</v>
       </c>
       <c r="C157" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D157" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E157">
         <v>4000</v>
@@ -4351,13 +4279,13 @@
         <v>161</v>
       </c>
       <c r="B158" t="s">
-        <v>375</v>
+        <v>353</v>
       </c>
       <c r="C158" t="s">
-        <v>437</v>
+        <v>414</v>
       </c>
       <c r="D158" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E158">
         <v>7000</v>
@@ -4368,13 +4296,13 @@
         <v>162</v>
       </c>
       <c r="B159" t="s">
-        <v>376</v>
+        <v>354</v>
       </c>
       <c r="C159" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D159" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E159">
         <v>5000</v>
@@ -4385,13 +4313,13 @@
         <v>163</v>
       </c>
       <c r="B160" t="s">
-        <v>377</v>
+        <v>355</v>
       </c>
       <c r="C160" t="s">
-        <v>437</v>
+        <v>414</v>
       </c>
       <c r="D160" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E160">
         <v>6000</v>
@@ -4402,13 +4330,13 @@
         <v>164</v>
       </c>
       <c r="B161" t="s">
-        <v>335</v>
+        <v>313</v>
       </c>
       <c r="C161" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D161" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E161">
         <v>5000</v>
@@ -4419,13 +4347,13 @@
         <v>165</v>
       </c>
       <c r="B162" t="s">
-        <v>362</v>
+        <v>340</v>
       </c>
       <c r="C162" t="s">
-        <v>437</v>
+        <v>414</v>
       </c>
       <c r="D162" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E162">
         <v>5000</v>
@@ -4436,13 +4364,13 @@
         <v>166</v>
       </c>
       <c r="B163" t="s">
-        <v>378</v>
+        <v>356</v>
       </c>
       <c r="C163" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D163" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E163">
         <v>7000</v>
@@ -4453,13 +4381,13 @@
         <v>167</v>
       </c>
       <c r="B164" t="s">
-        <v>369</v>
+        <v>347</v>
       </c>
       <c r="C164" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D164" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E164">
         <v>7000</v>
@@ -4470,13 +4398,13 @@
         <v>168</v>
       </c>
       <c r="B165" t="s">
-        <v>379</v>
+        <v>357</v>
       </c>
       <c r="C165" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D165" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E165">
         <v>4000</v>
@@ -4487,13 +4415,13 @@
         <v>169</v>
       </c>
       <c r="B166" t="s">
-        <v>362</v>
+        <v>340</v>
       </c>
       <c r="C166" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D166" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E166">
         <v>5000</v>
@@ -4504,13 +4432,13 @@
         <v>170</v>
       </c>
       <c r="B167" t="s">
-        <v>339</v>
+        <v>317</v>
       </c>
       <c r="C167" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D167" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E167">
         <v>7000</v>
@@ -4521,13 +4449,13 @@
         <v>171</v>
       </c>
       <c r="B168" t="s">
-        <v>311</v>
+        <v>289</v>
       </c>
       <c r="C168" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D168" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E168">
         <v>5000</v>
@@ -4538,13 +4466,13 @@
         <v>172</v>
       </c>
       <c r="B169" t="s">
-        <v>380</v>
+        <v>358</v>
       </c>
       <c r="C169" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D169" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E169">
         <v>7000</v>
@@ -4555,13 +4483,13 @@
         <v>173</v>
       </c>
       <c r="B170" t="s">
-        <v>351</v>
+        <v>329</v>
       </c>
       <c r="C170" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D170" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E170">
         <v>7000</v>
@@ -4572,13 +4500,13 @@
         <v>174</v>
       </c>
       <c r="B171" t="s">
-        <v>311</v>
+        <v>289</v>
       </c>
       <c r="C171" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="D171" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E171">
         <v>7000</v>
@@ -4589,13 +4517,13 @@
         <v>175</v>
       </c>
       <c r="B172" t="s">
-        <v>328</v>
+        <v>306</v>
       </c>
       <c r="C172" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D172" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E172">
         <v>7000</v>
@@ -4606,13 +4534,13 @@
         <v>176</v>
       </c>
       <c r="B173" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="C173" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D173" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E173">
         <v>5000</v>
@@ -4623,13 +4551,13 @@
         <v>177</v>
       </c>
       <c r="B174" t="s">
-        <v>364</v>
+        <v>342</v>
       </c>
       <c r="C174" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D174" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E174">
         <v>6000</v>
@@ -4640,13 +4568,13 @@
         <v>178</v>
       </c>
       <c r="B175" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C175" t="s">
-        <v>437</v>
+        <v>414</v>
       </c>
       <c r="D175" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E175">
         <v>7000</v>
@@ -4657,13 +4585,13 @@
         <v>179</v>
       </c>
       <c r="B176" t="s">
-        <v>307</v>
+        <v>285</v>
       </c>
       <c r="C176" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D176" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E176">
         <v>4000</v>
@@ -4674,13 +4602,13 @@
         <v>180</v>
       </c>
       <c r="B177" t="s">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="C177" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D177" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E177">
         <v>10000</v>
@@ -4691,13 +4619,13 @@
         <v>181</v>
       </c>
       <c r="B178" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C178" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D178" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E178">
         <v>8000</v>
@@ -4708,13 +4636,13 @@
         <v>182</v>
       </c>
       <c r="B179" t="s">
-        <v>311</v>
+        <v>289</v>
       </c>
       <c r="C179" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D179" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E179">
         <v>6000</v>
@@ -4725,13 +4653,13 @@
         <v>183</v>
       </c>
       <c r="B180" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C180" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D180" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E180">
         <v>7000</v>
@@ -4742,13 +4670,13 @@
         <v>184</v>
       </c>
       <c r="B181" t="s">
-        <v>381</v>
+        <v>359</v>
       </c>
       <c r="C181" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D181" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E181">
         <v>5000</v>
@@ -4759,13 +4687,13 @@
         <v>185</v>
       </c>
       <c r="B182" t="s">
-        <v>382</v>
+        <v>360</v>
       </c>
       <c r="C182" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D182" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E182">
         <v>6000</v>
@@ -4776,13 +4704,13 @@
         <v>186</v>
       </c>
       <c r="B183" t="s">
-        <v>383</v>
+        <v>361</v>
       </c>
       <c r="C183" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D183" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E183">
         <v>5000</v>
@@ -4793,13 +4721,13 @@
         <v>187</v>
       </c>
       <c r="B184" t="s">
-        <v>384</v>
+        <v>362</v>
       </c>
       <c r="C184" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D184" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E184">
         <v>7000</v>
@@ -4810,13 +4738,13 @@
         <v>188</v>
       </c>
       <c r="B185" t="s">
-        <v>385</v>
+        <v>363</v>
       </c>
       <c r="C185" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D185" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E185">
         <v>6000</v>
@@ -4827,13 +4755,13 @@
         <v>189</v>
       </c>
       <c r="B186" t="s">
-        <v>386</v>
+        <v>364</v>
       </c>
       <c r="C186" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D186" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E186">
         <v>6000</v>
@@ -4844,13 +4772,13 @@
         <v>190</v>
       </c>
       <c r="B187" t="s">
-        <v>387</v>
+        <v>365</v>
       </c>
       <c r="C187" t="s">
-        <v>425</v>
+        <v>402</v>
       </c>
       <c r="D187" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E187">
         <v>10000</v>
@@ -4861,13 +4789,13 @@
         <v>191</v>
       </c>
       <c r="B188" t="s">
-        <v>388</v>
+        <v>366</v>
       </c>
       <c r="C188" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D188" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E188">
         <v>8000</v>
@@ -4878,13 +4806,13 @@
         <v>192</v>
       </c>
       <c r="B189" t="s">
-        <v>349</v>
+        <v>327</v>
       </c>
       <c r="C189" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D189" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E189">
         <v>5000</v>
@@ -4895,13 +4823,13 @@
         <v>193</v>
       </c>
       <c r="B190" t="s">
-        <v>383</v>
+        <v>361</v>
       </c>
       <c r="C190" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D190" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E190">
         <v>5000</v>
@@ -4912,13 +4840,13 @@
         <v>194</v>
       </c>
       <c r="B191" t="s">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="C191" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D191" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E191">
         <v>5000</v>
@@ -4929,13 +4857,13 @@
         <v>195</v>
       </c>
       <c r="B192" t="s">
-        <v>341</v>
+        <v>319</v>
       </c>
       <c r="C192" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D192" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E192">
         <v>5000</v>
@@ -4946,13 +4874,13 @@
         <v>196</v>
       </c>
       <c r="B193" t="s">
-        <v>389</v>
+        <v>367</v>
       </c>
       <c r="C193" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D193" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E193">
         <v>8000</v>
@@ -4963,13 +4891,13 @@
         <v>197</v>
       </c>
       <c r="B194" t="s">
-        <v>383</v>
+        <v>361</v>
       </c>
       <c r="C194" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D194" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E194">
         <v>5000</v>
@@ -4980,13 +4908,13 @@
         <v>198</v>
       </c>
       <c r="B195" t="s">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="C195" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D195" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E195">
         <v>6000</v>
@@ -4997,13 +4925,13 @@
         <v>199</v>
       </c>
       <c r="B196" t="s">
-        <v>308</v>
+        <v>286</v>
       </c>
       <c r="C196" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D196" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E196">
         <v>5000</v>
@@ -5014,13 +4942,13 @@
         <v>200</v>
       </c>
       <c r="B197" t="s">
-        <v>383</v>
+        <v>361</v>
       </c>
       <c r="C197" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D197" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E197">
         <v>6000</v>
@@ -5031,13 +4959,13 @@
         <v>201</v>
       </c>
       <c r="B198" t="s">
-        <v>390</v>
+        <v>368</v>
       </c>
       <c r="C198" t="s">
-        <v>425</v>
+        <v>402</v>
       </c>
       <c r="D198" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E198">
         <v>10000</v>
@@ -5048,13 +4976,13 @@
         <v>202</v>
       </c>
       <c r="B199" t="s">
-        <v>391</v>
+        <v>369</v>
       </c>
       <c r="C199" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D199" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E199">
         <v>10000</v>
@@ -5065,13 +4993,13 @@
         <v>203</v>
       </c>
       <c r="B200" t="s">
-        <v>392</v>
+        <v>370</v>
       </c>
       <c r="C200" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D200" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E200">
         <v>10000</v>
@@ -5082,13 +5010,13 @@
         <v>204</v>
       </c>
       <c r="B201" t="s">
-        <v>393</v>
+        <v>371</v>
       </c>
       <c r="C201" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D201" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E201">
         <v>6000</v>
@@ -5099,13 +5027,13 @@
         <v>205</v>
       </c>
       <c r="B202" t="s">
-        <v>389</v>
+        <v>367</v>
       </c>
       <c r="C202" t="s">
-        <v>425</v>
+        <v>402</v>
       </c>
       <c r="D202" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E202">
         <v>7000</v>
@@ -5116,13 +5044,13 @@
         <v>206</v>
       </c>
       <c r="B203" t="s">
-        <v>394</v>
+        <v>372</v>
       </c>
       <c r="C203" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D203" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E203">
         <v>7000</v>
@@ -5133,13 +5061,13 @@
         <v>207</v>
       </c>
       <c r="B204" t="s">
-        <v>395</v>
+        <v>373</v>
       </c>
       <c r="C204" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D204" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E204">
         <v>7000</v>
@@ -5150,13 +5078,13 @@
         <v>208</v>
       </c>
       <c r="B205" t="s">
-        <v>396</v>
+        <v>374</v>
       </c>
       <c r="C205" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D205" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E205">
         <v>6000</v>
@@ -5167,13 +5095,13 @@
         <v>209</v>
       </c>
       <c r="B206" t="s">
-        <v>397</v>
+        <v>375</v>
       </c>
       <c r="C206" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D206" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E206">
         <v>7000</v>
@@ -5184,13 +5112,13 @@
         <v>210</v>
       </c>
       <c r="B207" t="s">
-        <v>307</v>
+        <v>285</v>
       </c>
       <c r="C207" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D207" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E207">
         <v>6000</v>
@@ -5201,13 +5129,13 @@
         <v>211</v>
       </c>
       <c r="B208" t="s">
-        <v>398</v>
+        <v>376</v>
       </c>
       <c r="C208" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D208" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E208">
         <v>7000</v>
@@ -5218,13 +5146,13 @@
         <v>212</v>
       </c>
       <c r="B209" t="s">
-        <v>399</v>
+        <v>377</v>
       </c>
       <c r="C209" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D209" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E209">
         <v>5000</v>
@@ -5235,13 +5163,13 @@
         <v>213</v>
       </c>
       <c r="B210" t="s">
-        <v>400</v>
+        <v>378</v>
       </c>
       <c r="C210" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D210" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E210">
         <v>10000</v>
@@ -5252,13 +5180,13 @@
         <v>214</v>
       </c>
       <c r="B211" t="s">
-        <v>401</v>
+        <v>379</v>
       </c>
       <c r="C211" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="D211" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E211">
         <v>6000</v>
@@ -5269,13 +5197,13 @@
         <v>215</v>
       </c>
       <c r="B212" t="s">
-        <v>398</v>
+        <v>376</v>
       </c>
       <c r="C212" t="s">
-        <v>435</v>
+        <v>412</v>
       </c>
       <c r="D212" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E212">
         <v>7000</v>
@@ -5286,13 +5214,13 @@
         <v>216</v>
       </c>
       <c r="B213" t="s">
-        <v>402</v>
+        <v>380</v>
       </c>
       <c r="C213" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D213" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E213">
         <v>6000</v>
@@ -5303,13 +5231,13 @@
         <v>217</v>
       </c>
       <c r="B214" t="s">
-        <v>403</v>
+        <v>381</v>
       </c>
       <c r="C214" t="s">
-        <v>425</v>
+        <v>402</v>
       </c>
       <c r="D214" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E214">
         <v>10000</v>
@@ -5320,13 +5248,13 @@
         <v>218</v>
       </c>
       <c r="B215" t="s">
+        <v>382</v>
+      </c>
+      <c r="C215" t="s">
         <v>404</v>
       </c>
-      <c r="C215" t="s">
-        <v>427</v>
-      </c>
       <c r="D215" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E215">
         <v>6000</v>
@@ -5337,13 +5265,13 @@
         <v>219</v>
       </c>
       <c r="B216" t="s">
-        <v>405</v>
+        <v>383</v>
       </c>
       <c r="C216" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D216" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E216">
         <v>5000</v>
@@ -5354,13 +5282,13 @@
         <v>220</v>
       </c>
       <c r="B217" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="C217" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D217" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E217">
         <v>7000</v>
@@ -5371,13 +5299,13 @@
         <v>221</v>
       </c>
       <c r="B218" t="s">
-        <v>406</v>
+        <v>384</v>
       </c>
       <c r="C218" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D218" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E218">
         <v>6000</v>
@@ -5388,13 +5316,13 @@
         <v>222</v>
       </c>
       <c r="B219" t="s">
-        <v>380</v>
+        <v>358</v>
       </c>
       <c r="C219" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D219" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E219">
         <v>7000</v>
@@ -5405,13 +5333,13 @@
         <v>223</v>
       </c>
       <c r="B220" t="s">
+        <v>385</v>
+      </c>
+      <c r="C220" t="s">
         <v>407</v>
       </c>
-      <c r="C220" t="s">
-        <v>430</v>
-      </c>
       <c r="D220" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E220">
         <v>5000</v>
@@ -5422,13 +5350,13 @@
         <v>224</v>
       </c>
       <c r="B221" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C221" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D221" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E221">
         <v>8000</v>
@@ -5439,13 +5367,13 @@
         <v>225</v>
       </c>
       <c r="B222" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="C222" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="D222" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E222">
         <v>5000</v>
@@ -5456,13 +5384,13 @@
         <v>226</v>
       </c>
       <c r="B223" t="s">
-        <v>408</v>
+        <v>386</v>
       </c>
       <c r="C223" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D223" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E223">
         <v>10000</v>
@@ -5473,13 +5401,13 @@
         <v>227</v>
       </c>
       <c r="B224" t="s">
-        <v>369</v>
+        <v>347</v>
       </c>
       <c r="C224" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D224" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E224">
         <v>6000</v>
@@ -5490,13 +5418,13 @@
         <v>228</v>
       </c>
       <c r="B225" t="s">
-        <v>311</v>
+        <v>289</v>
       </c>
       <c r="C225" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="D225" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E225">
         <v>7000</v>
@@ -5507,13 +5435,13 @@
         <v>229</v>
       </c>
       <c r="B226" t="s">
-        <v>409</v>
+        <v>387</v>
       </c>
       <c r="C226" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D226" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E226">
         <v>10000</v>
@@ -5524,13 +5452,13 @@
         <v>230</v>
       </c>
       <c r="B227" t="s">
-        <v>410</v>
+        <v>388</v>
       </c>
       <c r="C227" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D227" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E227">
         <v>8000</v>
@@ -5541,13 +5469,13 @@
         <v>231</v>
       </c>
       <c r="B228" t="s">
-        <v>307</v>
+        <v>285</v>
       </c>
       <c r="C228" t="s">
-        <v>437</v>
+        <v>414</v>
       </c>
       <c r="D228" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E228">
         <v>5000</v>
@@ -5558,13 +5486,13 @@
         <v>232</v>
       </c>
       <c r="B229" t="s">
-        <v>411</v>
+        <v>389</v>
       </c>
       <c r="C229" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D229" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E229">
         <v>10000</v>
@@ -5575,13 +5503,13 @@
         <v>233</v>
       </c>
       <c r="B230" t="s">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="C230" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D230" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E230">
         <v>10000</v>
@@ -5592,13 +5520,13 @@
         <v>234</v>
       </c>
       <c r="B231" t="s">
-        <v>412</v>
+        <v>390</v>
       </c>
       <c r="C231" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D231" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E231">
         <v>10000</v>
@@ -5609,13 +5537,13 @@
         <v>235</v>
       </c>
       <c r="B232" t="s">
-        <v>408</v>
+        <v>386</v>
       </c>
       <c r="C232" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D232" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E232">
         <v>8000</v>
@@ -5626,13 +5554,13 @@
         <v>236</v>
       </c>
       <c r="B233" t="s">
-        <v>413</v>
+        <v>391</v>
       </c>
       <c r="C233" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D233" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E233">
         <v>10000</v>
@@ -5643,13 +5571,13 @@
         <v>237</v>
       </c>
       <c r="B234" t="s">
-        <v>369</v>
+        <v>347</v>
       </c>
       <c r="C234" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D234" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E234">
         <v>8000</v>
@@ -5660,13 +5588,13 @@
         <v>238</v>
       </c>
       <c r="B235" t="s">
-        <v>414</v>
+        <v>392</v>
       </c>
       <c r="C235" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="D235" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E235">
         <v>10000</v>
@@ -5677,13 +5605,13 @@
         <v>239</v>
       </c>
       <c r="B236" t="s">
-        <v>415</v>
+        <v>393</v>
       </c>
       <c r="C236" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D236" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E236">
         <v>7000</v>
@@ -5694,13 +5622,13 @@
         <v>240</v>
       </c>
       <c r="B237" t="s">
+        <v>394</v>
+      </c>
+      <c r="C237" t="s">
+        <v>402</v>
+      </c>
+      <c r="D237" t="s">
         <v>416</v>
-      </c>
-      <c r="C237" t="s">
-        <v>425</v>
-      </c>
-      <c r="D237" t="s">
-        <v>439</v>
       </c>
       <c r="E237">
         <v>10000</v>
@@ -5711,13 +5639,13 @@
         <v>241</v>
       </c>
       <c r="B238" t="s">
-        <v>417</v>
+        <v>395</v>
       </c>
       <c r="C238" t="s">
-        <v>436</v>
+        <v>413</v>
       </c>
       <c r="D238" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E238">
         <v>8000</v>
@@ -5728,13 +5656,13 @@
         <v>242</v>
       </c>
       <c r="B239" t="s">
-        <v>312</v>
+        <v>290</v>
       </c>
       <c r="C239" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="D239" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E239">
         <v>5000</v>
@@ -5745,13 +5673,13 @@
         <v>243</v>
       </c>
       <c r="B240" t="s">
-        <v>335</v>
+        <v>313</v>
       </c>
       <c r="C240" t="s">
-        <v>437</v>
+        <v>414</v>
       </c>
       <c r="D240" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E240">
         <v>5000</v>
@@ -5762,13 +5690,13 @@
         <v>244</v>
       </c>
       <c r="B241" t="s">
-        <v>418</v>
+        <v>396</v>
       </c>
       <c r="C241" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D241" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="E241">
         <v>8000</v>
@@ -5779,13 +5707,13 @@
         <v>245</v>
       </c>
       <c r="B242" t="s">
-        <v>411</v>
+        <v>389</v>
       </c>
       <c r="C242" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="D242" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="E242">
         <v>6000</v>
@@ -5796,13 +5724,13 @@
         <v>246</v>
       </c>
       <c r="B243" t="s">
-        <v>390</v>
+        <v>368</v>
       </c>
       <c r="C243" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="D243" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E243">
         <v>10000</v>
@@ -5813,13 +5741,13 @@
         <v>247</v>
       </c>
       <c r="B244" t="s">
-        <v>419</v>
+        <v>397</v>
       </c>
       <c r="C244" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D244" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E244">
         <v>7000</v>
@@ -5830,13 +5758,13 @@
         <v>248</v>
       </c>
       <c r="B245" t="s">
-        <v>313</v>
+        <v>291</v>
       </c>
       <c r="C245" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="D245" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="E245">
         <v>10000</v>
@@ -5847,390 +5775,16 @@
         <v>249</v>
       </c>
       <c r="B246" t="s">
-        <v>301</v>
+        <v>279</v>
       </c>
       <c r="C246" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="D246" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="E246">
         <v>7000</v>
-      </c>
-    </row>
-    <row r="247" spans="1:5">
-      <c r="A247" t="s">
-        <v>250</v>
-      </c>
-      <c r="B247" t="s">
-        <v>420</v>
-      </c>
-      <c r="C247" t="s">
-        <v>420</v>
-      </c>
-      <c r="D247" t="s">
-        <v>442</v>
-      </c>
-      <c r="E247">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="248" spans="1:5">
-      <c r="A248" t="s">
-        <v>251</v>
-      </c>
-      <c r="B248" t="s">
-        <v>420</v>
-      </c>
-      <c r="C248" t="s">
-        <v>420</v>
-      </c>
-      <c r="D248" t="s">
-        <v>442</v>
-      </c>
-      <c r="E248">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="249" spans="1:5">
-      <c r="A249" t="s">
-        <v>252</v>
-      </c>
-      <c r="B249" t="s">
-        <v>420</v>
-      </c>
-      <c r="C249" t="s">
-        <v>420</v>
-      </c>
-      <c r="D249" t="s">
-        <v>442</v>
-      </c>
-      <c r="E249">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="250" spans="1:5">
-      <c r="A250" t="s">
-        <v>253</v>
-      </c>
-      <c r="B250" t="s">
-        <v>420</v>
-      </c>
-      <c r="C250" t="s">
-        <v>420</v>
-      </c>
-      <c r="D250" t="s">
-        <v>442</v>
-      </c>
-      <c r="E250">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="251" spans="1:5">
-      <c r="A251" t="s">
-        <v>254</v>
-      </c>
-      <c r="B251" t="s">
-        <v>420</v>
-      </c>
-      <c r="C251" t="s">
-        <v>420</v>
-      </c>
-      <c r="D251" t="s">
-        <v>442</v>
-      </c>
-      <c r="E251">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="252" spans="1:5">
-      <c r="A252" t="s">
-        <v>255</v>
-      </c>
-      <c r="B252" t="s">
-        <v>420</v>
-      </c>
-      <c r="C252" t="s">
-        <v>420</v>
-      </c>
-      <c r="D252" t="s">
-        <v>442</v>
-      </c>
-      <c r="E252">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="253" spans="1:5">
-      <c r="A253" t="s">
-        <v>256</v>
-      </c>
-      <c r="B253" t="s">
-        <v>420</v>
-      </c>
-      <c r="C253" t="s">
-        <v>420</v>
-      </c>
-      <c r="D253" t="s">
-        <v>442</v>
-      </c>
-      <c r="E253">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="254" spans="1:5">
-      <c r="A254" t="s">
-        <v>257</v>
-      </c>
-      <c r="B254" t="s">
-        <v>420</v>
-      </c>
-      <c r="C254" t="s">
-        <v>420</v>
-      </c>
-      <c r="D254" t="s">
-        <v>442</v>
-      </c>
-      <c r="E254">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="255" spans="1:5">
-      <c r="A255" t="s">
-        <v>258</v>
-      </c>
-      <c r="B255" t="s">
-        <v>420</v>
-      </c>
-      <c r="C255" t="s">
-        <v>420</v>
-      </c>
-      <c r="D255" t="s">
-        <v>442</v>
-      </c>
-      <c r="E255">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="256" spans="1:5">
-      <c r="A256" t="s">
-        <v>259</v>
-      </c>
-      <c r="B256" t="s">
-        <v>420</v>
-      </c>
-      <c r="C256" t="s">
-        <v>420</v>
-      </c>
-      <c r="D256" t="s">
-        <v>442</v>
-      </c>
-      <c r="E256">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="257" spans="1:5">
-      <c r="A257" t="s">
-        <v>260</v>
-      </c>
-      <c r="B257" t="s">
-        <v>420</v>
-      </c>
-      <c r="C257" t="s">
-        <v>420</v>
-      </c>
-      <c r="D257" t="s">
-        <v>442</v>
-      </c>
-      <c r="E257">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="258" spans="1:5">
-      <c r="A258" t="s">
-        <v>261</v>
-      </c>
-      <c r="B258" t="s">
-        <v>420</v>
-      </c>
-      <c r="C258" t="s">
-        <v>420</v>
-      </c>
-      <c r="D258" t="s">
-        <v>442</v>
-      </c>
-      <c r="E258">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="259" spans="1:5">
-      <c r="A259" t="s">
-        <v>262</v>
-      </c>
-      <c r="B259" t="s">
-        <v>420</v>
-      </c>
-      <c r="C259" t="s">
-        <v>420</v>
-      </c>
-      <c r="D259" t="s">
-        <v>442</v>
-      </c>
-      <c r="E259">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="260" spans="1:5">
-      <c r="A260" t="s">
-        <v>263</v>
-      </c>
-      <c r="B260" t="s">
-        <v>420</v>
-      </c>
-      <c r="C260" t="s">
-        <v>420</v>
-      </c>
-      <c r="D260" t="s">
-        <v>442</v>
-      </c>
-      <c r="E260">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="261" spans="1:5">
-      <c r="A261" t="s">
-        <v>264</v>
-      </c>
-      <c r="B261" t="s">
-        <v>420</v>
-      </c>
-      <c r="C261" t="s">
-        <v>420</v>
-      </c>
-      <c r="D261" t="s">
-        <v>442</v>
-      </c>
-      <c r="E261">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="262" spans="1:5">
-      <c r="A262" t="s">
-        <v>265</v>
-      </c>
-      <c r="B262" t="s">
-        <v>420</v>
-      </c>
-      <c r="C262" t="s">
-        <v>420</v>
-      </c>
-      <c r="D262" t="s">
-        <v>442</v>
-      </c>
-      <c r="E262">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="263" spans="1:5">
-      <c r="A263" t="s">
-        <v>266</v>
-      </c>
-      <c r="B263" t="s">
-        <v>420</v>
-      </c>
-      <c r="C263" t="s">
-        <v>420</v>
-      </c>
-      <c r="D263" t="s">
-        <v>442</v>
-      </c>
-      <c r="E263">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="264" spans="1:5">
-      <c r="A264" t="s">
-        <v>267</v>
-      </c>
-      <c r="B264" t="s">
-        <v>420</v>
-      </c>
-      <c r="C264" t="s">
-        <v>420</v>
-      </c>
-      <c r="D264" t="s">
-        <v>442</v>
-      </c>
-      <c r="E264">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="265" spans="1:5">
-      <c r="A265" t="s">
-        <v>268</v>
-      </c>
-      <c r="B265" t="s">
-        <v>420</v>
-      </c>
-      <c r="C265" t="s">
-        <v>420</v>
-      </c>
-      <c r="D265" t="s">
-        <v>442</v>
-      </c>
-      <c r="E265">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="266" spans="1:5">
-      <c r="A266" t="s">
-        <v>269</v>
-      </c>
-      <c r="B266" t="s">
-        <v>420</v>
-      </c>
-      <c r="C266" t="s">
-        <v>420</v>
-      </c>
-      <c r="D266" t="s">
-        <v>442</v>
-      </c>
-      <c r="E266">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="267" spans="1:5">
-      <c r="A267" t="s">
-        <v>270</v>
-      </c>
-      <c r="B267" t="s">
-        <v>420</v>
-      </c>
-      <c r="C267" t="s">
-        <v>420</v>
-      </c>
-      <c r="D267" t="s">
-        <v>442</v>
-      </c>
-      <c r="E267">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="268" spans="1:5">
-      <c r="A268" t="s">
-        <v>271</v>
-      </c>
-      <c r="B268" t="s">
-        <v>420</v>
-      </c>
-      <c r="C268" t="s">
-        <v>420</v>
-      </c>
-      <c r="D268" t="s">
-        <v>442</v>
-      </c>
-      <c r="E268">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>